<commit_message>
refactor and improve control
</commit_message>
<xml_diff>
--- a/files/304 Resistivity curve literature.xlsx
+++ b/files/304 Resistivity curve literature.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TDS\PycharmProjects\TDS_data_acquisition\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27AA6C0E-DB16-4AED-8679-68B827CC9D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A87970C-CE58-4CBF-87EE-FC705FD5C73D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -262,25 +262,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>2.7445385742069068</c:v>
+                  <c:v>0.82336157226207207</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.9539157437855783</c:v>
+                  <c:v>0.88617472313567336</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.0347546462052053</c:v>
+                  <c:v>1.2104263938615616</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.9118752214672066</c:v>
+                  <c:v>1.4735625664401619</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.3661977236758149</c:v>
+                  <c:v>1.9098593171027445</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7.152776820201094</c:v>
+                  <c:v>2.1458330460603281</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>7.3791305170429018</c:v>
+                  <c:v>2.21373915511287</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1439,13 +1439,13 @@
       </c>
       <c r="D3">
         <f>(C3/100000000)  * ($I$3/1000) /$H$7</f>
-        <v>2.7445385742069068</v>
+        <v>0.82336157226207207</v>
       </c>
       <c r="H3">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="I3">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="D4">
         <f t="shared" ref="D4:D9" si="0">(C4/100000000)  * ($I$3/1000) /$H$7</f>
-        <v>2.9539157437855783</v>
+        <v>0.88617472313567336</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>4.0347546462052053</v>
+        <v>1.2104263938615616</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="D6">
         <f t="shared" si="0"/>
-        <v>4.9118752214672066</v>
+        <v>1.4735625664401619</v>
       </c>
       <c r="H6" t="s">
         <v>8</v>
@@ -1496,11 +1496,11 @@
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>6.3661977236758149</v>
+        <v>1.9098593171027445</v>
       </c>
       <c r="H7">
         <f>(H3/1000000)^2 * PI() /4</f>
-        <v>1.7671458676442583E-8</v>
+        <v>7.0685834705770333E-8</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="D8">
         <f t="shared" si="0"/>
-        <v>7.152776820201094</v>
+        <v>2.1458330460603281</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="D9">
         <f t="shared" si="0"/>
-        <v>7.3791305170429018</v>
+        <v>2.21373915511287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>